<commit_message>
changes to fastpark report for plot visualisation and create of new prm report version for adjusmtent in month grouping logic
</commit_message>
<xml_diff>
--- a/output/FastPark_Report.xlsx
+++ b/output/FastPark_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onyx4-my.sharepoint.com/personal/jamie_douglas_edinburghairport_com/Documents/Documents/GitHub/EDI_airport_analytics/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_984D6DEF198874540B5FB6212ECD540AE079DB95" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83B20065-1008-4067-8283-0F24997891E1}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_984D6DEF198874540B5FB6212ECD540AE079DB95" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0773CB1A-800B-4DB4-85DA-648E83479302}"/>
   <bookViews>
-    <workbookView xWindow="21825" yWindow="3465" windowWidth="28905" windowHeight="15345" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19380" windowHeight="11320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly Movements" sheetId="1" r:id="rId1"/>
@@ -1848,10 +1848,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:C15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1862,7 +1862,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>10059</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>11426</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1895,7 +1895,7 @@
         <v>13420</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>13919</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -1917,7 +1917,7 @@
         <v>15615</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>15082</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1939,7 +1939,7 @@
         <v>14933</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>15156</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>16049</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>16974</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1983,7 +1983,7 @@
         <v>11814</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -1992,6 +1992,16 @@
       </c>
       <c r="C14">
         <v>9787</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B15">
+        <f>SUM(B3:B14)</f>
+        <v>165114</v>
+      </c>
+      <c r="C15">
+        <f>SUM(C3:C14)</f>
+        <v>164234</v>
       </c>
     </row>
   </sheetData>
@@ -2002,16 +2012,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:E25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="39.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" customWidth="1"/>
-    <col min="4" max="4" width="24.85546875" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="39.1796875" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="26.81640625" customWidth="1"/>
+    <col min="4" max="4" width="24.81640625" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -2028,7 +2038,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -2036,7 +2046,7 @@
         <v>168789</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2044,7 +2054,7 @@
         <v>165114</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -2052,7 +2062,7 @@
         <v>164234</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -2060,7 +2070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -2068,7 +2078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -2076,7 +2086,7 @@
         <v>28.586841272472459</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -2084,7 +2094,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -2092,7 +2102,7 @@
         <v>331799</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="C11" t="s">
         <v>28</v>
       </c>
@@ -2103,7 +2113,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="C12" t="s">
         <v>30</v>
       </c>
@@ -2114,7 +2124,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="C13" t="s">
         <v>32</v>
       </c>
@@ -2125,7 +2135,7 @@
         <v>1351</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -2133,7 +2143,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="15" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A15" t="s">
         <v>35</v>
       </c>
@@ -2141,7 +2151,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="16" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -2149,7 +2159,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -2157,7 +2167,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -2165,7 +2175,7 @@
         <v>-59941.683333333327</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -2173,7 +2183,7 @@
         <v>-5.8833333333333337</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -2181,7 +2191,7 @@
         <v>38.116666666666667</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>44</v>
       </c>
@@ -2189,7 +2199,7 @@
         <v>1668052.166666667</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>45</v>
       </c>
@@ -2197,7 +2207,7 @@
         <v>-525480</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>46</v>
       </c>
@@ -2205,7 +2215,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>47</v>
       </c>
@@ -2213,7 +2223,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -2229,12 +2239,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:N12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="14" max="14" width="11.28515625" customWidth="1"/>
+    <col min="14" max="14" width="11.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>49</v>
       </c>
@@ -2269,7 +2279,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>-99999</v>
       </c>
@@ -2305,7 +2315,7 @@
         <v>-180</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>-180</v>
       </c>
@@ -2341,7 +2351,7 @@
         <v>-120 to -180</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>-120</v>
       </c>
@@ -2377,7 +2387,7 @@
         <v>-60 to -120</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>-60</v>
       </c>
@@ -2413,7 +2423,7 @@
         <v>-30 to -60</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>-30</v>
       </c>
@@ -2449,7 +2459,7 @@
         <v>0 to -30</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>0</v>
       </c>
@@ -2485,7 +2495,7 @@
         <v>0 to 30</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>30</v>
       </c>
@@ -2521,7 +2531,7 @@
         <v>30 to 60</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>60</v>
       </c>
@@ -2557,7 +2567,7 @@
         <v>60 to 120</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>120</v>
       </c>
@@ -2593,7 +2603,7 @@
         <v>120 to 180</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>180</v>
       </c>
@@ -2637,14 +2647,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A2:C18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="17.7265625" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>60</v>
       </c>
@@ -2655,7 +2665,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>63</v>
       </c>
@@ -2666,7 +2676,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -2677,7 +2687,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>66</v>
       </c>
@@ -2688,7 +2698,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>67</v>
       </c>
@@ -2699,7 +2709,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>69</v>
       </c>
@@ -2710,7 +2720,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>70</v>
       </c>
@@ -2721,7 +2731,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -2732,7 +2742,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>73</v>
       </c>
@@ -2743,7 +2753,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>75</v>
       </c>
@@ -2754,7 +2764,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>76</v>
       </c>
@@ -2765,7 +2775,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>77</v>
       </c>
@@ -2776,7 +2786,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -2787,7 +2797,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>79</v>
       </c>
@@ -2798,7 +2808,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>80</v>
       </c>
@@ -2809,7 +2819,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>81</v>
       </c>
@@ -2820,7 +2830,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>82</v>
       </c>
@@ -2839,13 +2849,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A2:E46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="6" max="6" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>83</v>
       </c>
@@ -2859,7 +2869,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>87</v>
       </c>
@@ -2877,7 +2887,7 @@
         <v>23%</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>87</v>
       </c>
@@ -2895,7 +2905,7 @@
         <v>22%</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>87</v>
       </c>
@@ -2913,7 +2923,7 @@
         <v>8%</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>87</v>
       </c>
@@ -2927,7 +2937,7 @@
         <v>6.3108377915622462</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>87</v>
       </c>
@@ -2941,7 +2951,7 @@
         <v>2.7762472672982241</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>87</v>
       </c>
@@ -2955,7 +2965,7 @@
         <v>2.0670778309013031</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>87</v>
       </c>
@@ -2969,7 +2979,7 @@
         <v>1.8549787012186809</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>87</v>
       </c>
@@ -2983,7 +2993,7 @@
         <v>1.739449845665298</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>87</v>
       </c>
@@ -2997,7 +3007,7 @@
         <v>1.524980893304658</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>87</v>
       </c>
@@ -3011,7 +3021,7 @@
         <v>1.0332426876158991</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>87</v>
       </c>
@@ -3025,7 +3035,7 @@
         <v>1.010136916505223</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>87</v>
       </c>
@@ -3039,7 +3049,7 @@
         <v>0.99117833508107744</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>87</v>
       </c>
@@ -3053,7 +3063,7 @@
         <v>0.8928306939433257</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -3067,7 +3077,7 @@
         <v>0.86972492283264902</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>87</v>
       </c>
@@ -3081,7 +3091,7 @@
         <v>0.77433956004241988</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>87</v>
       </c>
@@ -3095,7 +3105,7 @@
         <v>0.62918792101381016</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>87</v>
       </c>
@@ -3109,7 +3119,7 @@
         <v>0.62741055400529655</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>87</v>
       </c>
@@ -3123,7 +3133,7 @@
         <v>0.39872266557654829</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>87</v>
       </c>
@@ -3137,7 +3147,7 @@
         <v>0.29563537908276022</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>87</v>
       </c>
@@ -3151,7 +3161,7 @@
         <v>0.26305031726001099</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>87</v>
       </c>
@@ -3165,7 +3175,7 @@
         <v>0.25594084922595672</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>87</v>
       </c>
@@ -3179,7 +3189,7 @@
         <v>0.25534839355645211</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>87</v>
       </c>
@@ -3193,7 +3203,7 @@
         <v>0.25238611520892951</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>87</v>
       </c>
@@ -3207,7 +3217,7 @@
         <v>0.23283507811528001</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>87</v>
       </c>
@@ -3221,7 +3231,7 @@
         <v>0.2109142183436124</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>87</v>
       </c>
@@ -3235,7 +3245,7 @@
         <v>0.20617457298757619</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>87</v>
       </c>
@@ -3249,7 +3259,7 @@
         <v>0.20380475030955811</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>87</v>
       </c>
@@ -3263,7 +3273,7 @@
         <v>0.16351776478325011</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>87</v>
       </c>
@@ -3277,7 +3287,7 @@
         <v>0.12619305760446481</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>87</v>
       </c>
@@ -3291,7 +3301,7 @@
         <v>0.10841938751932891</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>87</v>
       </c>
@@ -3305,7 +3315,7 @@
         <v>6.4577667975993694E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>87</v>
       </c>
@@ -3319,7 +3329,7 @@
         <v>4.7396453560362338E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>87</v>
       </c>
@@ -3333,7 +3343,7 @@
         <v>4.1471896865317062E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>87</v>
       </c>
@@ -3347,7 +3357,7 @@
         <v>3.791716284828988E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>87</v>
       </c>
@@ -3361,7 +3371,7 @@
         <v>3.7324707178785353E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>87</v>
       </c>
@@ -3375,7 +3385,7 @@
         <v>3.4362428831262698E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>87</v>
       </c>
@@ -3389,7 +3399,7 @@
         <v>2.0735948432658531E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>87</v>
       </c>
@@ -3403,7 +3413,7 @@
         <v>1.184911339009059E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>87</v>
       </c>
@@ -3417,7 +3427,7 @@
         <v>1.0664202051081531E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>87</v>
       </c>
@@ -3431,7 +3441,7 @@
         <v>2.3698226780181179E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>87</v>
       </c>
@@ -3445,7 +3455,7 @@
         <v>1.184911339009059E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>129</v>
       </c>
@@ -3459,7 +3469,7 @@
         <v>69.93939178500969</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>129</v>
       </c>
@@ -3473,7 +3483,7 @@
         <v>8.595939308841217</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>129</v>
       </c>
@@ -3495,16 +3505,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A2:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.140625" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" customWidth="1"/>
-    <col min="5" max="5" width="51.5703125" customWidth="1"/>
+    <col min="1" max="1" width="10.1796875" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" customWidth="1"/>
+    <col min="3" max="3" width="19.7265625" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" customWidth="1"/>
+    <col min="5" max="5" width="51.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>133</v>
       </c>
@@ -3518,7 +3528,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A3" s="16">
         <v>2025</v>
       </c>
@@ -3526,7 +3536,7 @@
         <v>168789</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="16">
         <v>2024</v>
       </c>
@@ -3540,7 +3550,7 @@
         <v>10.7961035039582</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="16">
         <v>2023</v>
       </c>
@@ -3554,7 +3564,7 @@
         <v>48.007295621750067</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2022</v>
       </c>
@@ -3568,7 +3578,7 @@
         <v>203.85058505850591</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="E8" s="15" t="str">
         <f>"FastPark Transactions " &amp; IF(D4&gt;=0, "grew by ", " decreased by ") &amp; TEXT(ABS(D4/100), "0.00%") &amp; " between " &amp; TEXT(A4, 0) &amp; " and " &amp; TEXT(A3, 0)</f>
         <v>FastPark Transactions grew by 10.80% between 2024 and 2025</v>
@@ -3582,7 +3592,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
final changes to PRM report for debugging and changes to fastpark graph
</commit_message>
<xml_diff>
--- a/output/FastPark_Report.xlsx
+++ b/output/FastPark_Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onyx4-my.sharepoint.com/personal/jamie_douglas_edinburghairport_com/Documents/Documents/GitHub/EDI_airport_analytics/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_984D6DEF198874540B5FB6212ECD540AE079DB95" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0773CB1A-800B-4DB4-85DA-648E83479302}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_984D6DEF198874540B5FB6212ECD540AE079DB95" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3F345D9-DD9B-4534-95E5-D01CDCF462AF}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19380" windowHeight="11320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="170" windowWidth="19380" windowHeight="11200" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly Movements" sheetId="1" r:id="rId1"/>
@@ -459,7 +459,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0,&quot;k&quot;"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -546,14 +546,6 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="6" tint="0.59999389629810485"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="16"/>
       <color theme="0" tint="-0.249977111117893"/>
       <name val="Calibri"/>
@@ -588,6 +580,38 @@
     <font>
       <sz val="11"/>
       <color theme="6" tint="0.59999389629810485"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FFD2B0C8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FFC1C1FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="6" tint="0.59999389629810485"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="0" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -653,7 +677,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -668,26 +692,34 @@
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFD2B0C8"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2143,11 +2175,11 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="15" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A15" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="23" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2159,11 +2191,11 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="17" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A17" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="24" t="s">
         <v>40</v>
       </c>
     </row>
@@ -2310,7 +2342,7 @@
       <c r="J3">
         <v>45</v>
       </c>
-      <c r="N3" s="23">
+      <c r="N3" s="22">
         <f>B3</f>
         <v>-180</v>
       </c>
@@ -2346,7 +2378,7 @@
       <c r="J4">
         <v>45</v>
       </c>
-      <c r="N4" s="23" t="str">
+      <c r="N4" s="22" t="str">
         <f>B4 &amp; " to " &amp; A4</f>
         <v>-120 to -180</v>
       </c>
@@ -2382,7 +2414,7 @@
       <c r="J5">
         <v>45</v>
       </c>
-      <c r="N5" s="23" t="str">
+      <c r="N5" s="22" t="str">
         <f>B5 &amp; " to " &amp; A5</f>
         <v>-60 to -120</v>
       </c>
@@ -2418,7 +2450,7 @@
       <c r="J6">
         <v>45</v>
       </c>
-      <c r="N6" s="23" t="str">
+      <c r="N6" s="22" t="str">
         <f>B6 &amp; " to " &amp; A6</f>
         <v>-30 to -60</v>
       </c>
@@ -2454,7 +2486,7 @@
       <c r="J7">
         <v>45</v>
       </c>
-      <c r="N7" s="23" t="str">
+      <c r="N7" s="22" t="str">
         <f>B7 &amp; " to " &amp; A7</f>
         <v>0 to -30</v>
       </c>
@@ -2490,7 +2522,7 @@
       <c r="J8">
         <v>45</v>
       </c>
-      <c r="N8" s="23" t="str">
+      <c r="N8" s="22" t="str">
         <f>A8 &amp; " to " &amp; B8</f>
         <v>0 to 30</v>
       </c>
@@ -2526,7 +2558,7 @@
       <c r="J9">
         <v>45</v>
       </c>
-      <c r="N9" s="23" t="str">
+      <c r="N9" s="22" t="str">
         <f>A9 &amp; " to " &amp; B9</f>
         <v>30 to 60</v>
       </c>
@@ -2562,7 +2594,7 @@
       <c r="J10">
         <v>45</v>
       </c>
-      <c r="N10" s="23" t="str">
+      <c r="N10" s="22" t="str">
         <f>A10 &amp; " to " &amp; B10</f>
         <v>60 to 120</v>
       </c>
@@ -2598,7 +2630,7 @@
       <c r="J11">
         <v>45</v>
       </c>
-      <c r="N11" s="23" t="str">
+      <c r="N11" s="22" t="str">
         <f>A11 &amp; " to " &amp; B11</f>
         <v>120 to 180</v>
       </c>
@@ -2634,7 +2666,7 @@
       <c r="J12">
         <v>45</v>
       </c>
-      <c r="N12" s="23" t="str">
+      <c r="N12" s="22" t="str">
         <f>A12 &amp; "+"</f>
         <v>180+</v>
       </c>
@@ -2873,7 +2905,7 @@
       <c r="A3" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>88</v>
       </c>
       <c r="C3">
@@ -2882,7 +2914,7 @@
       <c r="D3">
         <v>23.484350283490041</v>
       </c>
-      <c r="E3" s="20" t="str">
+      <c r="E3" s="19" t="str">
         <f>TEXT(D3, 0) &amp; "%"</f>
         <v>23%</v>
       </c>
@@ -2891,7 +2923,7 @@
       <c r="A4" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>89</v>
       </c>
       <c r="C4">
@@ -2900,7 +2932,7 @@
       <c r="D4">
         <v>21.96825622522795</v>
       </c>
-      <c r="E4" s="21" t="str">
+      <c r="E4" s="20" t="str">
         <f>TEXT(D4, 0) &amp; "%"</f>
         <v>22%</v>
       </c>
@@ -2909,7 +2941,7 @@
       <c r="A5" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>90</v>
       </c>
       <c r="C5">
@@ -2918,7 +2950,7 @@
       <c r="D5">
         <v>8.2860849936903467</v>
       </c>
-      <c r="E5" s="22" t="str">
+      <c r="E5" s="21" t="str">
         <f>TEXT(D5, 0) &amp; "%"</f>
         <v>8%</v>
       </c>
@@ -3528,19 +3560,19 @@
         <v>135</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="16">
+    <row r="3" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A3" s="15">
         <v>2025</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="25">
         <v>168789</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="16">
+    <row r="4" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A4" s="15">
         <v>2024</v>
       </c>
-      <c r="B4" s="14">
+      <c r="B4" s="26">
         <v>152342</v>
       </c>
       <c r="C4">
@@ -3551,10 +3583,10 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="16">
+      <c r="A5" s="15">
         <v>2023</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="13">
         <v>114041</v>
       </c>
       <c r="C5">
@@ -3579,7 +3611,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="E8" s="15" t="str">
+      <c r="E8" s="14" t="str">
         <f>"FastPark Transactions " &amp; IF(D4&gt;=0, "grew by ", " decreased by ") &amp; TEXT(ABS(D4/100), "0.00%") &amp; " between " &amp; TEXT(A4, 0) &amp; " and " &amp; TEXT(A3, 0)</f>
         <v>FastPark Transactions grew by 10.80% between 2024 and 2025</v>
       </c>

</xml_diff>

<commit_message>
changes to capex and SLA time
</commit_message>
<xml_diff>
--- a/output/FastPark_Report.xlsx
+++ b/output/FastPark_Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onyx4-my.sharepoint.com/personal/jamie_douglas_edinburghairport_com/Documents/Documents/GitHub/EDI_airport_analytics/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="11_984D6DEF198874540B5FB6212ECD540AE079DB95" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A7B30AD-80CB-4BA3-9A3C-07737461A09E}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_8F6405F84873C9CD4B1EA150DDF081C921A201F9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6C7DBD0-8AB6-45D9-857A-7CD68B005730}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly Movements" sheetId="1" r:id="rId1"/>
@@ -21,11 +21,8 @@
     <sheet name="Transaction Growth" sheetId="6" r:id="rId6"/>
     <sheet name="Charts" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -42,7 +39,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="121">
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Absolute Change</t>
+  </si>
+  <si>
+    <t>Percent Change</t>
+  </si>
   <si>
     <t>Month</t>
   </si>
@@ -53,40 +62,13 @@
     <t>Exits</t>
   </si>
   <si>
-    <t>2025-01</t>
-  </si>
-  <si>
-    <t>2025-02</t>
-  </si>
-  <si>
-    <t>2025-03</t>
-  </si>
-  <si>
-    <t>2025-04</t>
-  </si>
-  <si>
-    <t>2025-05</t>
-  </si>
-  <si>
-    <t>2025-06</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
   </si>
   <si>
     <t>Metric</t>
@@ -131,22 +113,25 @@
     <t>Peak Entries Day</t>
   </si>
   <si>
-    <t>24 May 2025</t>
+    <t>07 Feb 2026</t>
   </si>
   <si>
     <t>Peak Exits Day</t>
   </si>
   <si>
-    <t>19 Oct 2025</t>
+    <t>03 Jan 2026</t>
   </si>
   <si>
     <t>Peak Movements Day</t>
   </si>
   <si>
+    <t>14 Feb 2026</t>
+  </si>
+  <si>
     <t>Average Entry Difference (HH:MM)</t>
   </si>
   <si>
-    <t>00:54</t>
+    <t>01:22</t>
   </si>
   <si>
     <t>Median Entry Difference (HH:MM)</t>
@@ -158,13 +143,13 @@
     <t>Average Exit Difference (HH:MM)</t>
   </si>
   <si>
-    <t>02:14</t>
+    <t>09:42</t>
   </si>
   <si>
     <t>Median Exit Difference (HH:MM)</t>
   </si>
   <si>
-    <t>00:45</t>
+    <t>00:38</t>
   </si>
   <si>
     <t>Entry Min (mins)</t>
@@ -233,28 +218,28 @@
     <t>Kind</t>
   </si>
   <si>
-    <t>AXDGAJP5A</t>
+    <t>Z3OULUH</t>
   </si>
   <si>
     <t>Top 3</t>
   </si>
   <si>
-    <t>7L55C4KZ2</t>
-  </si>
-  <si>
-    <t>7JSM1BMF6</t>
-  </si>
-  <si>
-    <t>ZKPSPF9</t>
+    <t>LD751DR</t>
+  </si>
+  <si>
+    <t>AXF56QZER</t>
+  </si>
+  <si>
+    <t>AX88YV1AP</t>
   </si>
   <si>
     <t>Bottom 3</t>
   </si>
   <si>
-    <t>QXLSGMD</t>
-  </si>
-  <si>
-    <t>8ZM6VHT</t>
+    <t>8IU225NYK</t>
+  </si>
+  <si>
+    <t>AXP3AV068</t>
   </si>
   <si>
     <t>Average LOS</t>
@@ -299,21 +284,18 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Count</t>
-  </si>
-  <si>
     <t>Percent</t>
   </si>
   <si>
     <t>Airline</t>
   </si>
   <si>
+    <t>RYANAIR</t>
+  </si>
+  <si>
     <t>JET2</t>
   </si>
   <si>
-    <t>RYANAIR</t>
-  </si>
-  <si>
     <t>EASYJET</t>
   </si>
   <si>
@@ -326,111 +308,90 @@
     <t>QATAR AIRWAYS</t>
   </si>
   <si>
+    <t>KLM</t>
+  </si>
+  <si>
     <t>EMIRATES</t>
   </si>
   <si>
-    <t>KLM</t>
+    <t>UNITED AIRLINES</t>
+  </si>
+  <si>
+    <t>AIR FRANCE</t>
+  </si>
+  <si>
+    <t>TUI AIRWAYS</t>
+  </si>
+  <si>
+    <t>AER LINGUS</t>
+  </si>
+  <si>
+    <t>TURKISH AIRLINES</t>
+  </si>
+  <si>
+    <t>LUFTHANSA</t>
+  </si>
+  <si>
+    <t>LOGANAIR</t>
+  </si>
+  <si>
+    <t>PEGASUS AIRLINES</t>
+  </si>
+  <si>
+    <t>FINNAIR</t>
+  </si>
+  <si>
+    <t>EDELWEISS AIR</t>
+  </si>
+  <si>
+    <t>NORWEGIAN AIR SWEDEN</t>
+  </si>
+  <si>
+    <t>VUELING AIRLINES</t>
+  </si>
+  <si>
+    <t>ICELANDAIR</t>
+  </si>
+  <si>
+    <t>DELTA AIR LINES</t>
+  </si>
+  <si>
+    <t>AEGEAN AIRLINES</t>
+  </si>
+  <si>
+    <t>EUROWINGS</t>
   </si>
   <si>
     <t>SUNEXPRESS</t>
   </si>
   <si>
-    <t>UNITED AIRLINES</t>
-  </si>
-  <si>
-    <t>LUFTHANSA</t>
-  </si>
-  <si>
-    <t>LOGANAIR</t>
-  </si>
-  <si>
-    <t>AIR FRANCE</t>
-  </si>
-  <si>
-    <t>TURKISH AIRLINES</t>
-  </si>
-  <si>
-    <t>DELTA AIR LINES</t>
-  </si>
-  <si>
-    <t>AER LINGUS</t>
-  </si>
-  <si>
-    <t>VIRGIN ATLANTIC AIRWAYS</t>
-  </si>
-  <si>
-    <t>NORWEGIAN AIR SWEDEN</t>
+    <t>AMERICAN AIRLINES</t>
+  </si>
+  <si>
+    <t>HAINAN AIRLINES</t>
+  </si>
+  <si>
+    <t>BRUSSELS AIRLINES</t>
+  </si>
+  <si>
+    <t>AURIGNY AIR SERVICES</t>
+  </si>
+  <si>
+    <t>SAS</t>
+  </si>
+  <si>
+    <t>NORWEGIAN</t>
   </si>
   <si>
     <t>AIR CANADA</t>
   </si>
   <si>
-    <t>WESTJET</t>
-  </si>
-  <si>
-    <t>JETBLUE AIRWAYS</t>
-  </si>
-  <si>
-    <t>FINNAIR</t>
-  </si>
-  <si>
-    <t>EUROWINGS</t>
-  </si>
-  <si>
-    <t>PEGASUS AIRLINES</t>
-  </si>
-  <si>
-    <t>EDELWEISS AIR</t>
-  </si>
-  <si>
-    <t>AEGEAN AIRLINES</t>
-  </si>
-  <si>
-    <t>SAS</t>
-  </si>
-  <si>
-    <t>TUI AIRWAYS</t>
-  </si>
-  <si>
-    <t>VUELING AIRLINES</t>
-  </si>
-  <si>
-    <t>BRUSSELS AIRLINES</t>
+    <t>ASL AIRLINES FRANCE</t>
   </si>
   <si>
     <t>TRANSAVIA FRANCE</t>
   </si>
   <si>
-    <t>AMERICAN AIRLINES</t>
-  </si>
-  <si>
-    <t>HAINAN AIRLINES</t>
-  </si>
-  <si>
-    <t>AIREST CARGO</t>
-  </si>
-  <si>
-    <t>ATLANTIC AIRWAYS</t>
-  </si>
-  <si>
-    <t>ICELANDAIR</t>
-  </si>
-  <si>
-    <t>AURIGNY AIR SERVICES</t>
-  </si>
-  <si>
-    <t>AUSTRIAN AIRLINES</t>
-  </si>
-  <si>
-    <t>NORWEGIAN AIR INTERNATIONAL</t>
-  </si>
-  <si>
-    <t>LUFTHANSA CITY AIRLINES</t>
-  </si>
-  <si>
-    <t>NORWEGIAN</t>
-  </si>
-  <si>
     <t>Sector</t>
   </si>
   <si>
@@ -441,15 +402,6 @@
   </si>
   <si>
     <t>CTA</t>
-  </si>
-  <si>
-    <t>Period</t>
-  </si>
-  <si>
-    <t>Absolute Change</t>
-  </si>
-  <si>
-    <t>Percent Change</t>
   </si>
 </sst>
 </file>
@@ -716,10 +668,12 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -727,11 +681,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FFD2B0C8"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -854,38 +803,38 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>2011</c:v>
+                  <c:v>805</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5073</c:v>
+                  <c:v>1610</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>51369</c:v>
+                  <c:v>14594</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>67697</c:v>
+                  <c:v>13746</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20818</c:v>
+                  <c:v>3040</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13685</c:v>
+                  <c:v>2417</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2116</c:v>
+                  <c:v>646</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>445</c:v>
+                  <c:v>164</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>8</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F875-487F-BD04-DD58B6CAB074}"/>
+              <c16:uniqueId val="{00000000-BB4C-41E4-9878-2BDB21A44D21}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1000,6 +949,23 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Flight Info'!$B$37:$B$39</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>International</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Domestic</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>CTA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln>
               <a:noFill/>
@@ -1020,7 +986,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-BE6D-458A-A72D-5B03CFDB5090}"/>
+                <c16:uniqueId val="{00000001-AECC-4717-8270-65D95DE05BD3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1038,7 +1004,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-BE6D-458A-A72D-5B03CFDB5090}"/>
+                <c16:uniqueId val="{00000003-AECC-4717-8270-65D95DE05BD3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1056,7 +1022,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-BE6D-458A-A72D-5B03CFDB5090}"/>
+                <c16:uniqueId val="{00000005-AECC-4717-8270-65D95DE05BD3}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1102,7 +1068,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Flight Info'!$B$44:$B$46</c:f>
+              <c:f>'Flight Info'!$B$37:$B$39</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -1119,25 +1085,25 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Flight Info'!$C$44:$C$46</c:f>
+              <c:f>'Flight Info'!$C$37:$C$39</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>118050</c:v>
+                  <c:v>26981</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14509</c:v>
+                  <c:v>4993</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2680</c:v>
+                  <c:v>689</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000006-BE6D-458A-A72D-5B03CFDB5090}"/>
+              <c16:uniqueId val="{00000006-AECC-4717-8270-65D95DE05BD3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1352,41 +1318,41 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>2364</c:v>
+                  <c:v>475</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1476</c:v>
+                  <c:v>379</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8152</c:v>
+                  <c:v>1534</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>19928</c:v>
+                  <c:v>4116</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>72540</c:v>
+                  <c:v>16473</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>120736</c:v>
+                  <c:v>28799</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>65328</c:v>
+                  <c:v>14910</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>32367</c:v>
+                  <c:v>7073</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4549</c:v>
+                  <c:v>1029</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4346</c:v>
+                  <c:v>1041</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D200-4657-A7FD-4EFC975E5500}"/>
+              <c16:uniqueId val="{00000000-E069-4C9C-92EF-DA91200228B7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1892,160 +1858,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:C15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:C5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B3">
-        <v>8597</v>
+        <v>10130</v>
       </c>
       <c r="C3">
-        <v>10059</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>11674</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B4">
-        <v>12154</v>
+        <v>12174</v>
       </c>
       <c r="C4">
-        <v>11426</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>11745</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B5">
-        <v>14004</v>
+        <v>13740</v>
       </c>
       <c r="C5">
-        <v>13420</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>13726</v>
-      </c>
-      <c r="C6">
-        <v>13919</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
-        <v>16720</v>
-      </c>
-      <c r="C7">
-        <v>15615</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>15406</v>
-      </c>
-      <c r="C8">
-        <v>15082</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
-        <v>14872</v>
-      </c>
-      <c r="C9">
-        <v>14933</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10">
-        <v>14687</v>
-      </c>
-      <c r="C10">
-        <v>15156</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11">
-        <v>16275</v>
-      </c>
-      <c r="C11">
-        <v>16049</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12">
-        <v>15956</v>
-      </c>
-      <c r="C12">
-        <v>16974</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13">
-        <v>11370</v>
-      </c>
-      <c r="C13">
-        <v>11814</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14">
-        <v>11347</v>
-      </c>
-      <c r="C14">
-        <v>9787</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B15">
-        <f>SUM(B3:B14)</f>
-        <v>165114</v>
-      </c>
-      <c r="C15">
-        <f>SUM(C3:C14)</f>
-        <v>164234</v>
+        <v>14040</v>
       </c>
     </row>
   </sheetData>
@@ -2056,221 +1913,221 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:E25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="39.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" customWidth="1"/>
-    <col min="4" max="4" width="24.85546875" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" customWidth="1"/>
-    <col min="7" max="7" width="69.28515625" customWidth="1"/>
+    <col min="1" max="1" width="39.1796875" customWidth="1"/>
+    <col min="2" max="2" width="22.7265625" customWidth="1"/>
+    <col min="3" max="3" width="26.81640625" customWidth="1"/>
+    <col min="4" max="4" width="24.81640625" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="7" max="7" width="69.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A3" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" s="1">
+        <v>40192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>16</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B4">
+        <v>36044</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B5">
+        <v>37459</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>18</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="1">
-        <v>168789</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4">
-        <v>165114</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5">
-        <v>164234</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>23</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2">
+        <v>26.289508386960652</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>75837</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="4">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="C12" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="2">
-        <v>28.586841272472459</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="D12" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="E12" s="6">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="C13" t="s">
         <v>27</v>
       </c>
-      <c r="B10">
-        <v>331799</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="C11" t="s">
+      <c r="D13" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E13" s="8">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A14" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="4">
-        <v>853</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="C12" t="s">
+      <c r="B14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="5" t="s">
+    </row>
+    <row r="15" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A15" t="s">
         <v>31</v>
       </c>
-      <c r="E12" s="6">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="C13" t="s">
+      <c r="B15" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="8">
-        <v>1351</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A14" t="s">
+    </row>
+    <row r="16" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A16" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B16" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" t="s">
+    <row r="17" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A17" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B17" s="23" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A16" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B18">
+        <v>-44351.35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A17" t="s">
+      <c r="B19">
+        <v>-4.7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B20">
+        <v>37.283333333333331</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18">
-        <v>-59941.683333333327</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19">
-        <v>-5.8833333333333337</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20">
-        <v>38.116666666666667</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>44</v>
       </c>
       <c r="B21">
         <v>1668052.166666667</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B22">
-        <v>-525480</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>-397902</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B23">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B24">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B25">
         <v>2067995</v>
@@ -2284,48 +2141,48 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:P15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="14" max="14" width="11.28515625" customWidth="1"/>
-    <col min="16" max="16" width="36.28515625" customWidth="1"/>
+    <col min="14" max="14" width="11.26953125" customWidth="1"/>
+    <col min="16" max="16" width="36.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" t="s">
+      <c r="F2" t="s">
         <v>50</v>
       </c>
-      <c r="C2" t="s">
+      <c r="G2" t="s">
         <v>51</v>
       </c>
-      <c r="D2" t="s">
+      <c r="H2" t="s">
         <v>52</v>
       </c>
-      <c r="E2" t="s">
+      <c r="I2" t="s">
         <v>53</v>
       </c>
-      <c r="F2" t="s">
+      <c r="J2" t="s">
         <v>54</v>
       </c>
-      <c r="G2" t="s">
+      <c r="N2" t="s">
         <v>55</v>
       </c>
-      <c r="H2" t="s">
-        <v>56</v>
-      </c>
-      <c r="I2" t="s">
-        <v>57</v>
-      </c>
-      <c r="J2" t="s">
-        <v>58</v>
-      </c>
-      <c r="N2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>-99999</v>
       </c>
@@ -2336,32 +2193,32 @@
         <v>-50089.5</v>
       </c>
       <c r="D3">
-        <v>2364</v>
+        <v>475</v>
       </c>
       <c r="E3">
-        <v>1788</v>
+        <v>479</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H3">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I3">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J3">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N3" s="21">
         <f>B3</f>
         <v>-180</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>-180</v>
       </c>
@@ -2372,32 +2229,32 @@
         <v>-150</v>
       </c>
       <c r="D4">
-        <v>1476</v>
+        <v>379</v>
       </c>
       <c r="E4">
-        <v>295</v>
+        <v>85</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H4">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I4">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J4">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N4" s="21" t="str">
         <f>B4 &amp; " to " &amp; A4</f>
         <v>-120 to -180</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>-120</v>
       </c>
@@ -2408,32 +2265,32 @@
         <v>-90</v>
       </c>
       <c r="D5">
-        <v>8152</v>
+        <v>1534</v>
       </c>
       <c r="E5">
-        <v>455</v>
+        <v>104</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H5">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I5">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J5">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N5" s="21" t="str">
         <f>B5 &amp; " to " &amp; A5</f>
         <v>-60 to -120</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>-60</v>
       </c>
@@ -2444,32 +2301,32 @@
         <v>-45</v>
       </c>
       <c r="D6">
-        <v>19928</v>
+        <v>4116</v>
       </c>
       <c r="E6">
-        <v>357</v>
+        <v>129</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H6">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I6">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J6">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N6" s="21" t="str">
         <f>B6 &amp; " to " &amp; A6</f>
         <v>-30 to -60</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>-30</v>
       </c>
@@ -2480,32 +2337,32 @@
         <v>-15</v>
       </c>
       <c r="D7">
-        <v>72540</v>
+        <v>16473</v>
       </c>
       <c r="E7">
-        <v>3051</v>
+        <v>1494</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
       <c r="G7">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H7">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I7">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J7">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N7" s="21" t="str">
         <f>B7 &amp; " to " &amp; A7</f>
         <v>0 to -30</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>0</v>
       </c>
@@ -2516,32 +2373,32 @@
         <v>15</v>
       </c>
       <c r="D8">
-        <v>120736</v>
+        <v>28799</v>
       </c>
       <c r="E8">
-        <v>42382</v>
+        <v>12926</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H8">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I8">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J8">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N8" s="21" t="str">
         <f>A8 &amp; " to " &amp; B8</f>
         <v>0 to 30</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>30</v>
       </c>
@@ -2552,32 +2409,32 @@
         <v>45</v>
       </c>
       <c r="D9">
-        <v>65328</v>
+        <v>14910</v>
       </c>
       <c r="E9">
-        <v>63722</v>
+        <v>14345</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H9">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I9">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J9">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N9" s="21" t="str">
         <f>A9 &amp; " to " &amp; B9</f>
         <v>30 to 60</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>60</v>
       </c>
@@ -2588,32 +2445,32 @@
         <v>90</v>
       </c>
       <c r="D10">
-        <v>32367</v>
+        <v>7073</v>
       </c>
       <c r="E10">
-        <v>41209</v>
+        <v>7601</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H10">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I10">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J10">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N10" s="21" t="str">
         <f>A10 &amp; " to " &amp; B10</f>
         <v>60 to 120</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>120</v>
       </c>
@@ -2624,32 +2481,32 @@
         <v>150</v>
       </c>
       <c r="D11">
-        <v>4549</v>
+        <v>1029</v>
       </c>
       <c r="E11">
-        <v>7105</v>
+        <v>1165</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
       <c r="G11">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H11">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I11">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J11">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N11" s="21" t="str">
         <f>A11 &amp; " to " &amp; B11</f>
         <v>120 to 180</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>180</v>
       </c>
@@ -2660,39 +2517,39 @@
         <v>50089.5</v>
       </c>
       <c r="D12">
-        <v>4346</v>
+        <v>1041</v>
       </c>
       <c r="E12">
-        <v>7984</v>
+        <v>1818</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="G12">
-        <v>54.369208246055557</v>
+        <v>82.631132195730927</v>
       </c>
       <c r="H12">
-        <v>14.31666666666667</v>
+        <v>14.35</v>
       </c>
       <c r="I12">
-        <v>134.79540662695331</v>
+        <v>582.64906909597767</v>
       </c>
       <c r="J12">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="N12" s="21" t="str">
         <f>A12 &amp; "+"</f>
         <v>180+</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="60.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P14" s="28" t="str">
+    <row r="14" spans="1:16" ht="61" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P14" s="27" t="str">
         <f>"The majority of fastpark users will check-in "&amp; TEXT(ABS(H3), 0) &amp; " minutes " &amp; IF(H3 &lt;0, " earlier ", "later ") &amp; "than their booked entry time" &amp; " &amp; check-out " &amp; TEXT(ABS(J3), 0) &amp; " minutes " &amp; IF(J3 &lt;0, " earlier ", "later ") &amp; "than their booked exit time"</f>
-        <v>The majority of fastpark users will check-in 14 minutes later than their booked entry time &amp; check-out 45 minutes later than their booked exit time</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P15" s="27"/>
+        <v>The majority of fastpark users will check-in 14 minutes later than their booked entry time &amp; check-out 38 minutes later than their booked exit time</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="29.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="P15" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2702,198 +2559,198 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A2:C18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="17.7265625" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3">
+        <v>89.226342592592587</v>
+      </c>
+      <c r="C3" t="s">
         <v>60</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>61</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B4">
+        <v>83.852326388888883</v>
+      </c>
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B5">
+        <v>75.662997685185189</v>
+      </c>
+      <c r="C5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>63</v>
       </c>
-      <c r="B3">
-        <v>85.888483796296299</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B6">
+        <v>8.4953703703703701E-3</v>
+      </c>
+      <c r="C6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>65</v>
       </c>
-      <c r="B4">
-        <v>78.536759259259256</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B7">
+        <v>1.3032407407407409E-2</v>
+      </c>
+      <c r="C7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>66</v>
       </c>
-      <c r="B5">
-        <v>78.075046296296293</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B8">
+        <v>1.381944444444444E-2</v>
+      </c>
+      <c r="C8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="9" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.7">
+      <c r="A9" t="s">
         <v>67</v>
       </c>
-      <c r="B6">
-        <v>1.041666666666667E-4</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B9" s="11">
+        <v>7.388901963174205</v>
+      </c>
+      <c r="C9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>69</v>
       </c>
-      <c r="B7">
-        <v>3.7037037037037041E-4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B10">
+        <v>805</v>
+      </c>
+      <c r="C10" t="s">
         <v>70</v>
       </c>
-      <c r="B8">
-        <v>6.5972222222222224E-4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="31.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="11">
-        <v>7.9214878535051652</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B11">
+        <v>1610</v>
+      </c>
+      <c r="C11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B12">
+        <v>14594</v>
+      </c>
+      <c r="C12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>73</v>
       </c>
-      <c r="B10">
-        <v>2011</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="B13">
+        <v>13746</v>
+      </c>
+      <c r="C13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B14">
+        <v>3040</v>
+      </c>
+      <c r="C14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>75</v>
       </c>
-      <c r="B11">
-        <v>5073</v>
-      </c>
-      <c r="C11" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B15">
+        <v>2417</v>
+      </c>
+      <c r="C15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>76</v>
       </c>
-      <c r="B12">
-        <v>51369</v>
-      </c>
-      <c r="C12" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B16">
+        <v>646</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>77</v>
       </c>
-      <c r="B13">
-        <v>67697</v>
-      </c>
-      <c r="C13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B17">
+        <v>164</v>
+      </c>
+      <c r="C17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>78</v>
       </c>
-      <c r="B14">
-        <v>20818</v>
-      </c>
-      <c r="C14" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15">
-        <v>13685</v>
-      </c>
-      <c r="C15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>80</v>
-      </c>
-      <c r="B16">
-        <v>2116</v>
-      </c>
-      <c r="C16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17">
-        <v>445</v>
-      </c>
-      <c r="C17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>82</v>
-      </c>
       <c r="B18">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -2903,653 +2760,555 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A2:E46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:E39"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="6" max="6" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>88</v>
-      </c>
       <c r="C3">
-        <v>39639</v>
+        <v>7592</v>
       </c>
       <c r="D3">
-        <v>23.484350283490041</v>
+        <v>18.889331210191081</v>
       </c>
       <c r="E3" s="18" t="str">
         <f>TEXT(D3, 0) &amp; "%"</f>
-        <v>23%</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>19%</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C4">
-        <v>37080</v>
+        <v>7590</v>
       </c>
       <c r="D4">
-        <v>21.96825622522795</v>
+        <v>18.884355095541402</v>
       </c>
       <c r="E4" s="19" t="str">
         <f>TEXT(D4, 0) &amp; "%"</f>
-        <v>22%</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>19%</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C5">
-        <v>13986</v>
+        <v>7427</v>
       </c>
       <c r="D5">
-        <v>8.2860849936903467</v>
+        <v>18.478801751592361</v>
       </c>
       <c r="E5" s="20" t="str">
         <f>TEXT(D5, 0) &amp; "%"</f>
-        <v>8%</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>18%</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6">
+        <v>3106</v>
+      </c>
+      <c r="D6">
+        <v>7.7279060509554149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" t="s">
         <v>87</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C7">
+        <v>936</v>
+      </c>
+      <c r="D7">
+        <v>2.3288216560509549</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8">
+        <v>908</v>
+      </c>
+      <c r="D8">
+        <v>2.2591560509554141</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C9">
+        <v>771</v>
+      </c>
+      <c r="D9">
+        <v>1.9182921974522289</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10">
+        <v>770</v>
+      </c>
+      <c r="D10">
+        <v>1.9158041401273891</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" t="s">
         <v>91</v>
       </c>
-      <c r="C6">
-        <v>10652</v>
-      </c>
-      <c r="D6">
-        <v>6.3108377915622462</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="C11">
+        <v>513</v>
+      </c>
+      <c r="D11">
+        <v>1.276373407643312</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" t="s">
         <v>92</v>
       </c>
-      <c r="C7">
-        <v>4686</v>
-      </c>
-      <c r="D7">
-        <v>2.7762472672982241</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>87</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C12">
+        <v>421</v>
+      </c>
+      <c r="D12">
+        <v>1.047472133757962</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" t="s">
         <v>93</v>
       </c>
-      <c r="C8">
-        <v>3489</v>
-      </c>
-      <c r="D8">
-        <v>2.0670778309013031</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C13">
+        <v>393</v>
+      </c>
+      <c r="D13">
+        <v>0.97780652866242046</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" t="s">
         <v>94</v>
       </c>
-      <c r="C9">
-        <v>3131</v>
-      </c>
-      <c r="D9">
-        <v>1.8549787012186809</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C14">
+        <v>349</v>
+      </c>
+      <c r="D14">
+        <v>0.86833200636942687</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
         <v>95</v>
       </c>
-      <c r="C10">
-        <v>2936</v>
-      </c>
-      <c r="D10">
-        <v>1.739449845665298</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>87</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C15">
+        <v>342</v>
+      </c>
+      <c r="D15">
+        <v>0.85091560509554143</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" t="s">
         <v>96</v>
       </c>
-      <c r="C11">
-        <v>2574</v>
-      </c>
-      <c r="D11">
-        <v>1.524980893304658</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C16">
+        <v>322</v>
+      </c>
+      <c r="D16">
+        <v>0.80115445859872614</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" t="s">
         <v>97</v>
       </c>
-      <c r="C12">
-        <v>1744</v>
-      </c>
-      <c r="D12">
-        <v>1.0332426876158991</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>87</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C17">
+        <v>266</v>
+      </c>
+      <c r="D17">
+        <v>0.66182324840764339</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" t="s">
         <v>98</v>
       </c>
-      <c r="C13">
-        <v>1705</v>
-      </c>
-      <c r="D13">
-        <v>1.010136916505223</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="C18">
+        <v>176</v>
+      </c>
+      <c r="D18">
+        <v>0.43789808917197448</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" t="s">
         <v>99</v>
       </c>
-      <c r="C14">
-        <v>1673</v>
-      </c>
-      <c r="D14">
-        <v>0.99117833508107744</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>87</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C19">
+        <v>124</v>
+      </c>
+      <c r="D19">
+        <v>0.30851910828025481</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" t="s">
         <v>100</v>
       </c>
-      <c r="C15">
-        <v>1507</v>
-      </c>
-      <c r="D15">
-        <v>0.8928306939433257</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>87</v>
-      </c>
-      <c r="B16" t="s">
+      <c r="C20">
+        <v>105</v>
+      </c>
+      <c r="D20">
+        <v>0.26124601910828021</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" t="s">
         <v>101</v>
       </c>
-      <c r="C16">
-        <v>1468</v>
-      </c>
-      <c r="D16">
-        <v>0.86972492283264902</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>87</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="C21">
+        <v>99</v>
+      </c>
+      <c r="D21">
+        <v>0.24631767515923569</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" t="s">
         <v>102</v>
       </c>
-      <c r="C17">
-        <v>1307</v>
-      </c>
-      <c r="D17">
-        <v>0.77433956004241988</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>87</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C22">
+        <v>73</v>
+      </c>
+      <c r="D22">
+        <v>0.1816281847133758</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" t="s">
         <v>103</v>
       </c>
-      <c r="C18">
-        <v>1062</v>
-      </c>
-      <c r="D18">
-        <v>0.62918792101381016</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" t="s">
+      <c r="C23">
+        <v>71</v>
+      </c>
+      <c r="D23">
+        <v>0.17665207006369429</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>82</v>
+      </c>
+      <c r="B24" t="s">
         <v>104</v>
       </c>
-      <c r="C19">
-        <v>1059</v>
-      </c>
-      <c r="D19">
-        <v>0.62741055400529655</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="C24">
+        <v>65</v>
+      </c>
+      <c r="D24">
+        <v>0.16172372611464969</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" t="s">
         <v>105</v>
       </c>
-      <c r="C20">
-        <v>673</v>
-      </c>
-      <c r="D20">
-        <v>0.39872266557654829</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>87</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="C25">
+        <v>62</v>
+      </c>
+      <c r="D25">
+        <v>0.1542595541401274</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" t="s">
         <v>106</v>
       </c>
-      <c r="C21">
-        <v>499</v>
-      </c>
-      <c r="D21">
-        <v>0.29563537908276022</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>87</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="C26">
+        <v>42</v>
+      </c>
+      <c r="D26">
+        <v>0.1044984076433121</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>82</v>
+      </c>
+      <c r="B27" t="s">
         <v>107</v>
       </c>
-      <c r="C22">
-        <v>444</v>
-      </c>
-      <c r="D22">
-        <v>0.26305031726001099</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>87</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="C27">
+        <v>36</v>
+      </c>
+      <c r="D27">
+        <v>8.9570063694267524E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" t="s">
         <v>108</v>
       </c>
-      <c r="C23">
-        <v>432</v>
-      </c>
-      <c r="D23">
-        <v>0.25594084922595672</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>87</v>
-      </c>
-      <c r="B24" t="s">
+      <c r="C28">
+        <v>31</v>
+      </c>
+      <c r="D28">
+        <v>7.7129777070063701E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" t="s">
         <v>109</v>
       </c>
-      <c r="C24">
-        <v>431</v>
-      </c>
-      <c r="D24">
-        <v>0.25534839355645211</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>87</v>
-      </c>
-      <c r="B25" t="s">
+      <c r="C29">
+        <v>28</v>
+      </c>
+      <c r="D29">
+        <v>6.96656050955414E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>82</v>
+      </c>
+      <c r="B30" t="s">
         <v>110</v>
       </c>
-      <c r="C25">
-        <v>426</v>
-      </c>
-      <c r="D25">
-        <v>0.25238611520892951</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>87</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="C30">
+        <v>16</v>
+      </c>
+      <c r="D30">
+        <v>3.9808917197452227E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>82</v>
+      </c>
+      <c r="B31" t="s">
         <v>111</v>
       </c>
-      <c r="C26">
-        <v>393</v>
-      </c>
-      <c r="D26">
-        <v>0.23283507811528001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>87</v>
-      </c>
-      <c r="B27" t="s">
+      <c r="C31">
+        <v>11</v>
+      </c>
+      <c r="D31">
+        <v>2.7368630573248409E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" t="s">
         <v>112</v>
       </c>
-      <c r="C27">
-        <v>356</v>
-      </c>
-      <c r="D27">
-        <v>0.2109142183436124</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>87</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="C32">
+        <v>11</v>
+      </c>
+      <c r="D32">
+        <v>2.7368630573248409E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>82</v>
+      </c>
+      <c r="B33" t="s">
         <v>113</v>
       </c>
-      <c r="C28">
-        <v>348</v>
-      </c>
-      <c r="D28">
-        <v>0.20617457298757619</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>87</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="C33">
+        <v>3</v>
+      </c>
+      <c r="D33">
+        <v>7.4641719745222931E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" t="s">
         <v>114</v>
       </c>
-      <c r="C29">
-        <v>344</v>
-      </c>
-      <c r="D29">
-        <v>0.20380475030955811</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>87</v>
-      </c>
-      <c r="B30" t="s">
+      <c r="C34">
+        <v>2</v>
+      </c>
+      <c r="D34">
+        <v>4.9761146496815293E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>82</v>
+      </c>
+      <c r="B35" t="s">
         <v>115</v>
       </c>
-      <c r="C30">
-        <v>276</v>
-      </c>
-      <c r="D30">
-        <v>0.16351776478325011</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>87</v>
-      </c>
-      <c r="B31" t="s">
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35">
+        <v>2.4880573248407651E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>82</v>
+      </c>
+      <c r="B36" t="s">
         <v>116</v>
       </c>
-      <c r="C31">
-        <v>213</v>
-      </c>
-      <c r="D31">
-        <v>0.12619305760446481</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>87</v>
-      </c>
-      <c r="B32" t="s">
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <v>2.4880573248407651E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>117</v>
       </c>
-      <c r="C32">
-        <v>183</v>
-      </c>
-      <c r="D32">
-        <v>0.10841938751932891</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>87</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="B37" t="s">
         <v>118</v>
       </c>
-      <c r="C33">
-        <v>109</v>
-      </c>
-      <c r="D33">
-        <v>6.4577667975993694E-2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>87</v>
-      </c>
-      <c r="B34" t="s">
+      <c r="C37">
+        <v>26981</v>
+      </c>
+      <c r="D37">
+        <v>67.130274681528661</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B38" t="s">
         <v>119</v>
       </c>
-      <c r="C34">
-        <v>80</v>
-      </c>
-      <c r="D34">
-        <v>4.7396453560362338E-2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B35" t="s">
+      <c r="C38">
+        <v>4993</v>
+      </c>
+      <c r="D38">
+        <v>12.422870222929941</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>117</v>
+      </c>
+      <c r="B39" t="s">
         <v>120</v>
       </c>
-      <c r="C35">
-        <v>70</v>
-      </c>
-      <c r="D35">
-        <v>4.1471896865317062E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>87</v>
-      </c>
-      <c r="B36" t="s">
-        <v>121</v>
-      </c>
-      <c r="C36">
-        <v>64</v>
-      </c>
-      <c r="D36">
-        <v>3.791716284828988E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>87</v>
-      </c>
-      <c r="B37" t="s">
-        <v>122</v>
-      </c>
-      <c r="C37">
-        <v>63</v>
-      </c>
-      <c r="D37">
-        <v>3.7324707178785353E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>87</v>
-      </c>
-      <c r="B38" t="s">
-        <v>123</v>
-      </c>
-      <c r="C38">
-        <v>58</v>
-      </c>
-      <c r="D38">
-        <v>3.4362428831262698E-2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>87</v>
-      </c>
-      <c r="B39" t="s">
-        <v>124</v>
-      </c>
       <c r="C39">
-        <v>35</v>
+        <v>689</v>
       </c>
       <c r="D39">
-        <v>2.0735948432658531E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>87</v>
-      </c>
-      <c r="B40" t="s">
-        <v>125</v>
-      </c>
-      <c r="C40">
-        <v>20</v>
-      </c>
-      <c r="D40">
-        <v>1.184911339009059E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>87</v>
-      </c>
-      <c r="B41" t="s">
-        <v>126</v>
-      </c>
-      <c r="C41">
-        <v>18</v>
-      </c>
-      <c r="D41">
-        <v>1.0664202051081531E-2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>87</v>
-      </c>
-      <c r="B42" t="s">
-        <v>127</v>
-      </c>
-      <c r="C42">
-        <v>4</v>
-      </c>
-      <c r="D42">
-        <v>2.3698226780181179E-3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>87</v>
-      </c>
-      <c r="B43" t="s">
-        <v>128</v>
-      </c>
-      <c r="C43">
-        <v>2</v>
-      </c>
-      <c r="D43">
-        <v>1.184911339009059E-3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>129</v>
-      </c>
-      <c r="B44" t="s">
-        <v>130</v>
-      </c>
-      <c r="C44">
-        <v>118050</v>
-      </c>
-      <c r="D44">
-        <v>69.93939178500969</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>129</v>
-      </c>
-      <c r="B45" t="s">
-        <v>131</v>
-      </c>
-      <c r="C45">
-        <v>14509</v>
-      </c>
-      <c r="D45">
-        <v>8.595939308841217</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>129</v>
-      </c>
-      <c r="B46" t="s">
-        <v>132</v>
-      </c>
-      <c r="C46">
-        <v>2680</v>
-      </c>
-      <c r="D46">
-        <v>1.587781194272138</v>
+        <v>1.714271496815287</v>
       </c>
     </row>
   </sheetData>
@@ -3560,83 +3319,83 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A2:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.140625" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" customWidth="1"/>
-    <col min="5" max="5" width="59.85546875" customWidth="1"/>
+    <col min="1" max="1" width="10.1796875" customWidth="1"/>
+    <col min="2" max="2" width="14.1796875" customWidth="1"/>
+    <col min="3" max="3" width="19.7265625" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>134</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A3" s="14">
+        <v>2026</v>
+      </c>
+      <c r="B3" s="24">
+        <v>40192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A4" s="14">
         <v>2025</v>
       </c>
-      <c r="B3" s="24">
-        <v>168789</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="14">
+      <c r="B4" s="25">
+        <v>38428</v>
+      </c>
+      <c r="C4">
+        <v>1764</v>
+      </c>
+      <c r="D4">
+        <v>4.5904028312688663</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="14">
         <v>2024</v>
       </c>
-      <c r="B4" s="25">
-        <v>152342</v>
-      </c>
-      <c r="C4">
-        <v>16447</v>
-      </c>
-      <c r="D4">
-        <v>10.7961035039582</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="24.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="14">
+      <c r="B5" s="13">
+        <v>36507</v>
+      </c>
+      <c r="C5">
+        <v>3685</v>
+      </c>
+      <c r="D5">
+        <v>10.093954584052369</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A6">
         <v>2023</v>
       </c>
-      <c r="B5" s="13">
-        <v>114041</v>
-      </c>
-      <c r="C5">
-        <v>54748</v>
-      </c>
-      <c r="D5">
-        <v>48.007295621750067</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>2022</v>
-      </c>
       <c r="B6" s="12">
-        <v>55550</v>
+        <v>19394</v>
       </c>
       <c r="C6">
-        <v>113239</v>
+        <v>20798</v>
       </c>
       <c r="D6">
-        <v>203.85058505850591</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E8" s="26" t="str">
-        <f>"FastPark Transactions " &amp; IF(D4&gt;=0, "grew by ", " decreased by ") &amp; TEXT(ABS(D4/100), "0.00%") &amp; " between " &amp; TEXT(A4, 0) &amp; " and " &amp; TEXT(A3, 0)</f>
-        <v>FastPark Transactions grew by 10.80% between 2024 and 2025</v>
+        <v>107.23935237702381</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E8" s="28" t="str">
+        <f>"FastPark Transactions " &amp; IF(D4&gt;=0, "grew by ", " decreased by ") &amp; TEXT(ABS(D4/100), "0.00%") &amp; " for the same period between " &amp; TEXT(A4, 0) &amp; " and " &amp; TEXT(A3, 0)</f>
+        <v>FastPark Transactions grew by 4.59% for the same period between 2025 and 2026</v>
       </c>
     </row>
   </sheetData>
@@ -3647,7 +3406,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>